<commit_message>
Clarify World Map wording and mark it as an illustrative Claude-made map
Rewrites the World Map tab text: new title and kicker, a highlighted
notice that the map and codes were created with Claude from a
ChatGPT-generated dataset and are a teaching illustration rather than
research, a 'What the map shows' paragraph, a 'How to read it' list,
a revised empty detail card, and a footer on provenance plus a class
discussion prompt. The '+' variants are now described as fused with
theocratic or religious-nationalist claims rather than 'religion'.

The workbook gets the same notice at the top of Methodology, records
the ChatGPT origin of the base dataset in Sources and the leader-source
note, updates the C+ and RE+ definitions, and logs the change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VZNCsVwvMc2u2uycCR1cma
</commit_message>
<xml_diff>
--- a/Freedenian_Ideologies_Global_Dataset_2026-10-03.xlsx
+++ b/Freedenian_Ideologies_Global_Dataset_2026-10-03.xlsx
@@ -15,9 +15,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'195 States'!$A$1:$M$196</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Methodology'!$A$1:$B$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sources'!$A$1:$C$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Change log'!$A$1:$F$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Methodology'!$A$1:$B$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sources'!$A$1:$C$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Change log'!$A$1:$F$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,12 +46,17 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE2D6"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -66,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -75,6 +80,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -12687,7 +12695,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Conservative core combined strongly with nationalism, populism, religion or authoritarianism.</t>
+          <t>Conservative core combined strongly with nationalism, populism, religious-nationalist claims or authoritarian rule.</t>
         </is>
       </c>
     </row>
@@ -12843,7 +12851,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Religious legitimacy fused with dynastic or national authority.</t>
+          <t>Theocratic claims to legitimacy fused with dynastic or national authority.</t>
         </is>
       </c>
     </row>
@@ -13050,7 +13058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -13070,355 +13078,367 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Snapshot date</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03 (leaders as in the corrected conservatism dataset of the same date)</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Created with Claude. Illustrative only.</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>This dataset's ideological codes were created with Claude (Anthropic's AI model), starting from a dataset generated with ChatGPT. It is a representative teaching illustration, not the result of actual research. Treat every code as material to question, not as evidence.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Coverage</t>
+          <t>Snapshot date</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>195 states: 193 UN members + Palestine + Vatican City. Country names follow UN short names.</t>
+          <t>2026-10-03 (leaders as in the corrected conservatism dataset of the same date)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Leader source</t>
+          <t>Coverage</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Wikipedia list of current heads of state and government (retrieved 2026-10-03), cross-checked against news reports. Unchanged from the source dataset.</t>
+          <t>195 states: 193 UN members + Palestine + Vatican City. Country names follow UN short names.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Framework</t>
+          <t>Leader source</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Michael Freeden's morphological approach: an ideology is a configuration of core, adjacent and peripheral concepts, each 'decontested' (given one settled meaning). Families are identified by their core concepts, not by a left-right position or a checklist of policies. Each family appears in several decontested variants.</t>
+          <t>Heads of state and government are taken from the ChatGPT-generated source dataset, which states that they follow the Wikipedia list of current heads of state and government (retrieved 2026-10-03), cross-checked against news reports. They have not been independently verified for this revision.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Unit coded</t>
+          <t>Framework</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The governing ideology of the executive that actually directs policy (normally the head of government, or the head of state where executive power sits there). A ceremonial head of state does not determine the code.</t>
+          <t>Michael Freeden's morphological approach: an ideology is a configuration of core, adjacent and peripheral concepts, each 'decontested' (given one settled meaning). Families are identified by their core concepts, not by a left-right position or a checklist of policies. Each family appears in several decontested variants.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Ideological family</t>
+          <t>Unit coded</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>The macro-ideology whose core concepts organise the government's programme: Liberalism, Conservatism, Socialism, plus Religious-political ideology and a residual Traditionalist-authoritarian category. Nationalism is never coded as the family: in Freeden's account it is thin-centred and needs a host, so it is recorded as a component (and signalled by "+" variants).</t>
+          <t>The governing ideology of the executive that actually directs policy (normally the head of government, or the head of state where executive power sits there). A ceremonial head of state does not determine the code.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Liberalism</t>
+          <t>Ideological family</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Core concepts (Freeden): liberty, rationality, individuality, progress, sociability, the general interest, and limited, accountable power.</t>
+          <t>The macro-ideology whose core concepts organise the government's programme: Liberalism, Conservatism, Socialism, plus Religious-political ideology and a residual Traditionalist-authoritarian category. Nationalism is never coded as the family: in Freeden's account it is thin-centred and needs a host, so it is recorded as a component (and signalled by "+" variants).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Conservatism</t>
+          <t>Liberalism</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Core concepts (Freeden): change must be controlled so that it appears natural and organic; social order has extra-human origins (history, God, nature, the market or monarchy) and is independent of human will.</t>
+          <t>Core concepts (Freeden): liberty, rationality, individuality, progress, sociability, the general interest, and limited, accountable power.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Socialism</t>
+          <t>Conservatism</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Core concepts (Freeden): the constitutive nature of the group, equality, human welfare as the goal of politics, human activity/praxis, and history as the arena of change.</t>
+          <t>Core concepts (Freeden): change must be controlled so that it appears natural and organic; social order has extra-human origins (history, God, nature, the market or monarchy) and is independent of human will.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Religious-political ideology</t>
+          <t>Socialism</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Political order is derived from religious doctrine and religious authority. Not one of Freeden's three macro-ideologies; included because his morphological method treats such belief systems as ideologies with their own core concepts (divine sovereignty, sacred law, clerical or dynastic-religious authority).</t>
+          <t>Core concepts (Freeden): the constitutive nature of the group, equality, human welfare as the goal of politics, human activity/praxis, and history as the arena of change.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Traditionalist-authoritarian</t>
+          <t>Religious-political ideology</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Residual category, not a Freeden family: hierarchy, order, continuity and state authority dominate, but no liberal, conservative or socialist programme is sustained at the core. Typical of military, personalist and dominant-party regimes. Calling these conservative would overstate the presence of conservative morphology; nationalism usually appears as a component.</t>
+          <t>Political order is derived from religious doctrine and religious authority. Not one of Freeden's three macro-ideologies; included because his morphological method treats such belief systems as ideologies with their own core concepts (divine sovereignty, sacred law, clerical or dynastic-religious authority).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>L - Liberalism</t>
+          <t>Traditionalist-authoritarian</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Clear liberal morphology: social, market or centrist liberalism.</t>
+          <t>Residual category, not a Freeden family: hierarchy, order, continuity and state authority dominate, but no liberal, conservative or socialist programme is sustained at the core. Typical of military, personalist and dominant-party regimes. Calling these conservative would overstate the presence of conservative morphology; nationalism usually appears as a component.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>L+ - National / populist liberalism</t>
+          <t>L - Liberalism</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Liberal core combined strongly with nationalism or populism.</t>
+          <t>Clear liberal morphology: social, market or centrist liberalism.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>C - Conservatism</t>
+          <t>L+ - National / populist liberalism</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Clear conservative morphology: Christian-democratic, liberal-conservative or customary conservatism.</t>
+          <t>Liberal core combined strongly with nationalism or populism.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>C+ - National / religious / populist conservatism</t>
+          <t>C - Conservatism</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Conservative core combined strongly with nationalism, populism, religion or authoritarianism.</t>
+          <t>Clear conservative morphology: Christian-democratic, liberal-conservative or customary conservatism.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Cm - Monarchical traditionalism</t>
+          <t>C+ - National / religious / populist conservatism</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>A ruling monarchy manages change from above to preserve a dynastic and often religious order.</t>
+          <t>Conservative core combined strongly with nationalism, populism, religious-nationalist claims or authoritarian rule.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>S - Social democracy</t>
+          <t>Cm - Monarchical traditionalism</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Social democracy or democratic socialism within a competitive democracy.</t>
+          <t>A ruling monarchy manages change from above to preserve a dynastic and often religious order.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>S+ - Left-nationalist / left-populist socialism</t>
+          <t>S - Social democracy</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Socialist core combined strongly with nationalism, populism or authoritarianism.</t>
+          <t>Social democracy or democratic socialism within a competitive democracy.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>SM - Marxism-Leninism</t>
+          <t>S+ - Left-nationalist / left-populist socialism</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Communist party-state; the party's doctrine organises state and economy.</t>
+          <t>Socialist core combined strongly with nationalism, populism or authoritarianism.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>RE - Theocracy</t>
+          <t>SM - Marxism-Leninism</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Religious doctrine and clerical authority define the state.</t>
+          <t>Communist party-state; the party's doctrine organises state and economy.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>RE+ - Religious-national rule</t>
+          <t>RE - Theocracy</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Religious legitimacy fused with dynastic or national authority.</t>
+          <t>Religious doctrine and clerical authority define the state.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>T - Traditionalist-authoritarian</t>
+          <t>RE+ - Religious-national rule</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Order, hierarchy and continuity without a sustained macro-ideology (military, personalist or dominant-party rule).</t>
+          <t>Theocratic claims to legitimacy fused with dynastic or national authority.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>The "+" variants</t>
+          <t>T - Traditionalist-authoritarian</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>As in the earlier conservatism scheme (C vs C+), "+" marks a family core combined strongly with a thin-centred ideology (nationalism, populism) or with religion or authoritarian rule. C+ is national/religious/populist conservatism, S+ left-nationalist or left-populist socialism, L+ national or populist liberalism, RE+ religious-national rule.</t>
+          <t>Order, hierarchy and continuity without a sustained macro-ideology (military, personalist or dominant-party rule).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Secondary family</t>
+          <t>The "+" variants</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>A second family whose core concepts are clearly present in adjacent positions (e.g. coalition partners). Written VARIANT/SECONDARY, e.g. C/LIB = conservatism with liberal adjacency, T/SOC = traditionalist-authoritarian rule with a socialist legacy.</t>
+          <t>As in the earlier conservatism scheme (C vs C+), "+" marks a family core combined strongly with a thin-centred ideology (nationalism, populism), with theocratic or religious-nationalist claims, or with authoritarian rule. C+ is national/religious/populist conservatism, S+ left-nationalist or left-populist socialism, L+ national or populist liberalism, RE+ religious-national rule.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Thin-centred components</t>
+          <t>Secondary family</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Freeden's thin-centred ideologies that attach to a host: Nationalism, Populism (people vs. elite; see also Mudde 2004), Ecologism (green), Feminism. Listed where they visibly shape the governing programme.</t>
+          <t>A second family whose core concepts are clearly present in adjacent positions (e.g. coalition partners). Written VARIANT/SECONDARY, e.g. C/LIB = conservatism with liberal adjacency, T/SOC = traditionalist-authoritarian rule with a socialist legacy.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Adjacent concepts / regime context</t>
+          <t>Thin-centred components</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Religion and Developmentalism are recorded as adjacent concepts. Authoritarian rule is regime context, not an ideology: it is recorded so that students can separate how power is held from what ideas justify it.</t>
+          <t>Freeden's thin-centred ideologies that attach to a host: Nationalism, Populism (people vs. elite; see also Mudde 2004), Ecologism (green), Feminism. Listed where they visibly shape the governing programme.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Hard cases</t>
+          <t>Adjacent concepts / regime context</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Russia is coded C+ because "traditional values" conservatism is now official doctrine, not just regime practice. North Korea stays in the socialist family (SM) although Juche nationalism dominates its core. Ex-Marxist dominant parties (Angola, Mozambique, Tanzania, Eritrea, Zimbabwe, Republic of the Congo) are coded T with SOC as secondary family, because socialism survives only as a legacy.</t>
+          <t>Religion and Developmentalism are recorded as adjacent concepts. Authoritarian rule is regime context, not an ideology: it is recorded so that students can separate how power is held from what ideas justify it.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Previous code</t>
+          <t>Hard cases</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>The final column keeps the code from the conservatism-only scheme (C, C+, L/C, R, T and hybrids) so the two classifications can be compared.</t>
+          <t>Russia is coded C+ because "traditional values" conservatism is now official doctrine, not just regime practice. North Korea stays in the socialist family (SM) although Juche nationalism dominates its core. Ex-Marxist dominant parties (Angola, Mozambique, Tanzania, Eritrea, Zimbabwe, Republic of the Congo) are coded T with SOC as secondary family, because socialism survives only as a legacy.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>Previous code</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>The final column keeps the code from the conservatism-only scheme (C, C+, L/C, R, T and hybrids) so the two classifications can be compared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>Caveat</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Codes are interpretive judgements for teaching and discussion, not measurements. Coalitions, caretaker and transitional governments are coded by their dominant governing morphology. The policy column is descriptive and unchanged from the source dataset.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B30"/>
+  <autoFilter ref="A1:B31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13429,7 +13449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -13457,68 +13477,64 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Current leaders</t>
+          <t>Base dataset</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>UN Protocol &amp; Liaison Service</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.un.org/dgacm/en/content/protocol/hshgnfa</t>
-        </is>
-      </c>
+          <t>Freedenian Conservatism Global Dataset (snapshot 2026-10-03, corrected), generated with ChatGPT and supplied for this course; ideological codes revised with Claude.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Current leaders cross-check</t>
+          <t>Current leaders</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>CIA World Leaders</t>
+          <t>UN Protocol &amp; Liaison Service</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>https://www.cia.gov/resources/world-leaders/</t>
+          <t>https://www.un.org/dgacm/en/content/protocol/hshgnfa</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Current heads list used for 2026 snapshot</t>
+          <t>Current leaders cross-check</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Wikipedia – List of current heads of state and government</t>
+          <t>CIA World Leaders</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/List_of_current_heads_of_state_and_government</t>
+          <t>https://www.cia.gov/resources/world-leaders/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Freeden framework</t>
+          <t>Current heads list used for 2026 snapshot</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Stanford Encyclopedia of Philosophy – Conservatism</t>
+          <t>Wikipedia – List of current heads of state and government</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>https://seop.illc.uva.nl/entries/conservatism/</t>
+          <t>https://en.wikipedia.org/wiki/List_of_current_heads_of_state_and_government</t>
         </is>
       </c>
     </row>
@@ -13530,50 +13546,54 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Freeden, M. (1996) Ideologies and Political Theory: A Conceptual Approach. Oxford: Clarendon Press.</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n"/>
+          <t>Stanford Encyclopedia of Philosophy – Conservatism</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://seop.illc.uva.nl/entries/conservatism/</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Thin-centred nationalism</t>
+          <t>Freeden framework</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Freeden, M. (1998) "Is Nationalism a Distinct Ideology?" Political Studies 46(4): 748-765.</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1111/1467-9248.00165</t>
-        </is>
-      </c>
+          <t>Freeden, M. (1996) Ideologies and Political Theory: A Conceptual Approach. Oxford: Clarendon Press.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Freeden framework (introductory)</t>
+          <t>Thin-centred nationalism</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Freeden, M. (2003) Ideology: A Very Short Introduction. Oxford: Oxford University Press.</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n"/>
+          <t>Freeden, M. (1998) "Is Nationalism a Distinct Ideology?" Political Studies 46(4): 748-765.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/1467-9248.00165</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Families and variants</t>
+          <t>Freeden framework (introductory)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Freeden, M., Sargent, L.T. and Stears, M. (eds) (2013) The Oxford Handbook of Political Ideologies. Oxford: Oxford University Press.</t>
+          <t>Freeden, M. (2003) Ideology: A Very Short Introduction. Oxford: Oxford University Press.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n"/>
@@ -13581,22 +13601,35 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Families and variants</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Freeden, M., Sargent, L.T. and Stears, M. (eds) (2013) The Oxford Handbook of Political Ideologies. Oxford: Oxford University Press.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Thin-centred populism</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Mudde, C. (2004) "The Populist Zeitgeist." Government and Opposition 39(4): 541-563.</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/j.1477-7053.2004.00135.x</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C10"/>
+  <autoFilter ref="A1:C11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13607,7 +13640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F111"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13653,7 +13686,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Recoding</t>
+          <t>Notice</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -13663,22 +13696,22 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>Methodology</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Five families with nationalism as a possible primary family (LIB, CON, SOC, NAT, REL)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Variants within each family (L, L+; C, C+, Cm; S, S+, SM; RE, RE+) plus residual T; nationalism only as a component</t>
+          <t>"Created with Claude. Illustrative only." notice; ChatGPT origin of the base dataset recorded; "+" variants worded as theocratic or religious-nationalist claims rather than religion</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Nationalism is thin-centred (Freeden 1998) and is not treated as a host ideology; variants show the range of decontested forms within each family, as C and C+ did in the conservatism scheme</t>
+          <t>Clarify provenance and that the dataset is a teaching illustration, not research</t>
         </is>
       </c>
     </row>
@@ -13690,7 +13723,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>All 195 states</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -13700,17 +13733,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>NAT/SOC</t>
+          <t>Five families with nationalism as a possible primary family (LIB, CON, SOC, NAT, REL)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>S+</t>
+          <t>Variants within each family (L, L+; C, C+, Cm; S, S+, SM; RE, RE+) plus residual T; nationalism only as a component</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Former NAT-primary state reassigned to the family whose core concepts it draws on, or to the residual T category</t>
+          <t>Nationalism is thin-centred (Freeden 1998) and is not treated as a host ideology; variants show the range of decontested forms within each family, as C and C+ did in the conservatism scheme</t>
         </is>
       </c>
     </row>
@@ -13722,7 +13755,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Angola</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -13737,7 +13770,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>T/SOC</t>
+          <t>S+</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -13754,7 +13787,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Azerbaijan</t>
+          <t>Angola</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -13764,12 +13797,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/SOC</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T/SOC</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -13786,7 +13819,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>Azerbaijan</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -13796,12 +13829,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>NAT/CON</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -13818,7 +13851,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Belarus</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -13833,7 +13866,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>T/SOC</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -13850,7 +13883,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Belarus</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -13860,12 +13893,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>NAT/LIB</t>
+          <t>NAT/CON</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>C+/SOC</t>
+          <t>T/SOC</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -13882,7 +13915,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -13892,12 +13925,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>NAT/SOC</t>
+          <t>NAT/LIB</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>S+</t>
+          <t>C+/SOC</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -13914,7 +13947,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Burkina Faso</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -13946,7 +13979,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Burundi</t>
+          <t>Burkina Faso</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -13956,12 +13989,12 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/SOC</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>S+</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -13978,7 +14011,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>Burundi</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -13988,12 +14021,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>NAT/CON</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>T/CON</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -14010,7 +14043,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Cameroon</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -14025,7 +14058,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T/CON</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -14042,7 +14075,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Central African Republic</t>
+          <t>Cameroon</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -14052,7 +14085,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/CON</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -14074,7 +14107,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Chad</t>
+          <t>Central African Republic</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -14106,7 +14139,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Comoros</t>
+          <t>Chad</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -14116,12 +14149,12 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>NAT/REL</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>T/REL</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -14138,7 +14171,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Comoros</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -14148,12 +14181,12 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>NAT/CON</t>
+          <t>NAT/REL</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>T/REL</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -14170,7 +14203,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Djibouti</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -14180,12 +14213,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/CON</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -14202,7 +14235,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Djibouti</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -14234,7 +14267,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>El Salvador</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -14244,12 +14277,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>NAT/CON</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -14266,7 +14299,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Equatorial Guinea</t>
+          <t>El Salvador</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -14276,12 +14309,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/CON</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -14298,7 +14331,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Eritrea</t>
+          <t>Equatorial Guinea</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -14308,12 +14341,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>NAT/SOC</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>T/SOC</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -14330,7 +14363,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Ethiopia</t>
+          <t>Eritrea</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -14340,12 +14373,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>NAT/LIB</t>
+          <t>NAT/SOC</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>T/LIB</t>
+          <t>T/SOC</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -14362,7 +14395,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Gabon</t>
+          <t>Ethiopia</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -14372,12 +14405,12 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/LIB</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T/LIB</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -14394,7 +14427,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Gabon</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -14404,12 +14437,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>NAT/CON</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -14426,7 +14459,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Guinea</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -14436,12 +14469,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/CON</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -14458,7 +14491,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Guinea-Bissau</t>
+          <t>Guinea</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -14490,7 +14523,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Guinea-Bissau</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -14500,12 +14533,12 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>NAT/CON</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -14522,7 +14555,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -14554,7 +14587,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -14586,7 +14619,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -14596,12 +14629,12 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/CON</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -14618,7 +14651,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -14628,12 +14661,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>NAT/CON</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>T/CON</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -14650,7 +14683,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Libya</t>
+          <t>Kyrgyzstan</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -14660,12 +14693,12 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>NAT/LIB</t>
+          <t>NAT/CON</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>T/LIB</t>
+          <t>T/CON</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -14682,7 +14715,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Madagascar</t>
+          <t>Libya</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -14692,12 +14725,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/LIB</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T/LIB</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -14714,7 +14747,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Maldives</t>
+          <t>Madagascar</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -14724,12 +14757,12 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>NAT/REL</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -14746,7 +14779,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Mali</t>
+          <t>Maldives</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -14756,12 +14789,12 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/REL</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -14778,7 +14811,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Mauritania</t>
+          <t>Mali</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -14788,12 +14821,12 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>NAT/REL</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>T/REL</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -14810,7 +14843,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Mozambique</t>
+          <t>Mauritania</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -14820,12 +14853,12 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>NAT/SOC</t>
+          <t>NAT/REL</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>T/SOC</t>
+          <t>T/REL</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -14842,7 +14875,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Myanmar</t>
+          <t>Mozambique</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -14852,12 +14885,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>NAT/REL</t>
+          <t>NAT/SOC</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>T/REL</t>
+          <t>T/SOC</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -14874,7 +14907,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Nicaragua</t>
+          <t>Myanmar</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -14884,12 +14917,12 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>NAT/SOC</t>
+          <t>NAT/REL</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>S+</t>
+          <t>T/REL</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -14906,7 +14939,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Niger</t>
+          <t>Nicaragua</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -14916,12 +14949,12 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/SOC</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>S+</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -14938,7 +14971,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>North Korea</t>
+          <t>Niger</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -14948,12 +14981,12 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>NAT/SOC</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>SM</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -14970,7 +15003,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>North Korea</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -14980,12 +15013,12 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>NAT/REL</t>
+          <t>NAT/SOC</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>SM</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -15002,7 +15035,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Palestine</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -15012,12 +15045,12 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/REL</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>S+</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -15034,7 +15067,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Republic of the Congo</t>
+          <t>Palestine</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -15044,12 +15077,12 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>NAT/SOC</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>T/SOC</t>
+          <t>S+</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -15066,7 +15099,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Republic of the Congo</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -15076,12 +15109,12 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>NAT/CON</t>
+          <t>NAT/SOC</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>T/SOC</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -15098,7 +15131,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Rwanda</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -15108,12 +15141,12 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/CON</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -15130,7 +15163,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Rwanda</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -15140,12 +15173,12 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>NAT/SOC</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>S+</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -15162,7 +15195,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -15172,12 +15205,12 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>NAT/CON</t>
+          <t>NAT/SOC</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>S+</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -15194,7 +15227,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -15204,12 +15237,12 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>NAT/SOC</t>
+          <t>NAT/CON</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>S+/CON</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -15226,7 +15259,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Somalia</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -15236,12 +15269,12 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>NAT/REL</t>
+          <t>NAT/SOC</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>T/REL</t>
+          <t>S+/CON</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -15258,7 +15291,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>South Sudan</t>
+          <t>Somalia</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -15268,12 +15301,12 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/REL</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>T/REL</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -15290,7 +15323,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Sudan</t>
+          <t>South Sudan</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -15322,7 +15355,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Tajikistan</t>
+          <t>Sudan</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -15354,7 +15387,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Tanzania</t>
+          <t>Tajikistan</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -15364,12 +15397,12 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>NAT/SOC</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>T/SOC</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -15386,7 +15419,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Timor-Leste</t>
+          <t>Tanzania</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -15396,12 +15429,12 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/SOC</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>L+</t>
+          <t>T/SOC</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -15418,7 +15451,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Togo</t>
+          <t>Timor-Leste</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -15433,7 +15466,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>L+</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -15450,7 +15483,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Togo</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -15482,7 +15515,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Turkmenistan</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -15514,7 +15547,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Uganda</t>
+          <t>Turkmenistan</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -15524,12 +15557,12 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>NAT/CON</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>T/CON</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -15546,7 +15579,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Uganda</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -15561,7 +15594,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>C+</t>
+          <t>T/CON</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -15578,7 +15611,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Uzbekistan</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -15588,12 +15621,12 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/CON</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -15610,7 +15643,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Yemen</t>
+          <t>Uzbekistan</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -15620,12 +15653,12 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>NAT/REL</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>T/REL</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -15642,7 +15675,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Yemen</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -15652,12 +15685,12 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NAT/REL</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>T/SOC</t>
+          <t>T/REL</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -15674,7 +15707,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>All 195 states</t>
+          <t>Zimbabwe</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -15684,17 +15717,17 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Conservatism-only scheme (C, C+, L/C, R, T)</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Freeden ideological families (LIB, CON, SOC, NAT, REL) + secondary family + thin-centred components</t>
+          <t>T/SOC</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Dataset broadened from "how conservative is this government?" to "which ideological family organises it?"; previous code retained in the last column</t>
+          <t>Former NAT-primary state reassigned to the family whose core concepts it draws on, or to the residual T category</t>
         </is>
       </c>
     </row>
@@ -15706,7 +15739,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>All 195 states</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -15716,17 +15749,17 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>R - centre-right security-oriented</t>
+          <t>Conservatism-only scheme (C, C+, L/C, R, T)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>SOC/NAT - social democracy (LSDP-led coalition)</t>
+          <t>Freeden ideological families (LIB, CON, SOC, NAT, REL) + secondary family + thin-centred components</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Prime Minister Sinkevičius leads the Social Democratic Party (LSDP); previous R code did not match the governing party</t>
+          <t>Dataset broadened from "how conservative is this government?" to "which ideological family organises it?"; previous code retained in the last column</t>
         </is>
       </c>
     </row>
@@ -15738,7 +15771,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>T-coded states (39)</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -15748,17 +15781,17 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>T - traditionalist-authoritarian</t>
+          <t>R - centre-right security-oriented</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>NAT, CON (monarchical traditionalism) or REL</t>
+          <t>SOC/NAT - social democracy (LSDP-led coalition)</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>The residual T category is not a Freeden family; split by the core concepts that organise each regime</t>
+          <t>Prime Minister Sinkevičius leads the Social Democratic Party (LSDP); previous R code did not match the governing party</t>
         </is>
       </c>
     </row>
@@ -15770,7 +15803,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>L/C-coded states (59)</t>
+          <t>T-coded states (39)</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -15780,81 +15813,81 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>L/C</t>
+          <t>T - traditionalist-authoritarian</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>LIB or SOC (social democracy) by governing party, NAT where liberation/developmental nationalism dominates</t>
+          <t>NAT, CON (monarchical traditionalism) or REL</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>L/C merged liberal and socialist governments; Freeden treats liberalism and socialism as distinct macro-ideologies</t>
+          <t>The residual T category is not a Freeden family; split by the core concepts that organise each regime</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Factual</t>
+          <t>Recoding</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>L/C-coded states (59)</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Head of state</t>
+          <t>Classification</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Mohammed Shahabuddin</t>
+          <t>L/C</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Mirza Fakhrul Islam Alamgir</t>
+          <t>LIB or SOC (social democracy) by governing party, NAT where liberation/developmental nationalism dominates</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Shahabuddin resigned 24 Jul 2026; Alamgir elected 20 Aug 2026</t>
+          <t>L/C merged liberal and socialist governments; Freeden treats liberalism and socialism as distinct macro-ideologies</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>C/L split</t>
+          <t>Factual</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>Head of state</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>C/L — centre-right liberal</t>
+          <t>Mohammed Shahabuddin</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>R — centre-right liberal</t>
+          <t>Mirza Fakhrul Islam Alamgir</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
+          <t>Shahabuddin resigned 24 Jul 2026; Alamgir elected 20 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -15866,7 +15899,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -15876,17 +15909,17 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>C/L — fragmented coalition</t>
+          <t>C/L — centre-right liberal</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>L/C — fragmented coalition</t>
+          <t>R — centre-right liberal</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
+          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
         </is>
       </c>
     </row>
@@ -15898,7 +15931,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Congo, Democratic Republic of the</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -15908,12 +15941,12 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>C/L — centrist-developmental</t>
+          <t>C/L — fragmented coalition</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>L/C — centrist-developmental</t>
+          <t>L/C — fragmented coalition</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -15930,7 +15963,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Congo, Democratic Republic of the</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -15940,17 +15973,17 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>C/L — moderate centre-right</t>
+          <t>C/L — centrist-developmental</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>R — moderate centre-right</t>
+          <t>L/C — centrist-developmental</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
+          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
         </is>
       </c>
     </row>
@@ -15962,7 +15995,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Dominican Republic</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -15972,17 +16005,17 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>C/L — liberal-centrist, not primarily conservative</t>
+          <t>C/L — moderate centre-right</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>L/C — liberal-centrist, not primarily conservative</t>
+          <t>R — moderate centre-right</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
+          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
         </is>
       </c>
     </row>
@@ -15994,7 +16027,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Guyana</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -16004,12 +16037,12 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>C/L — developmental-centrist</t>
+          <t>C/L — liberal-centrist, not primarily conservative</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>L/C — developmental-centrist</t>
+          <t>L/C — liberal-centrist, not primarily conservative</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -16026,7 +16059,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Ivory Coast</t>
+          <t>Guyana</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -16036,17 +16069,17 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>C/L — developmental centre-right</t>
+          <t>C/L — developmental-centrist</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>R — developmental centre-right</t>
+          <t>L/C — developmental-centrist</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
+          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
         </is>
       </c>
     </row>
@@ -16058,7 +16091,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Kiribati</t>
+          <t>Ivory Coast</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -16068,17 +16101,17 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>C/L — developmental-centrist</t>
+          <t>C/L — developmental centre-right</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>L/C — developmental-centrist</t>
+          <t>R — developmental centre-right</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
+          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
         </is>
       </c>
     </row>
@@ -16090,7 +16123,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Kiribati</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -16100,17 +16133,17 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>C/L — centre-right liberal</t>
+          <t>C/L — developmental-centrist</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>R — centre-right liberal</t>
+          <t>L/C — developmental-centrist</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
+          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
         </is>
       </c>
     </row>
@@ -16122,7 +16155,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Lebanon</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -16132,17 +16165,17 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>C/L — institutional/coalitional</t>
+          <t>C/L — centre-right liberal</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>L/C — institutional/coalitional</t>
+          <t>R — centre-right liberal</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
+          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
         </is>
       </c>
     </row>
@@ -16154,7 +16187,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Lesotho</t>
+          <t>Lebanon</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -16164,17 +16197,17 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>C/L — centre-right developmental</t>
+          <t>C/L — institutional/coalitional</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>R — centre-right developmental</t>
+          <t>L/C — institutional/coalitional</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
+          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16219,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Libya</t>
+          <t>Lesotho</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -16196,17 +16229,17 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>C/L — fragmented transitional</t>
+          <t>C/L — centre-right developmental</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>L/C — fragmented transitional</t>
+          <t>R — centre-right developmental</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
+          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
         </is>
       </c>
     </row>
@@ -16218,7 +16251,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Libya</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -16228,17 +16261,17 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>C/L — centre-right security-oriented</t>
+          <t>C/L — fragmented transitional</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>R — centre-right security-oriented</t>
+          <t>L/C — fragmented transitional</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
+          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
         </is>
       </c>
     </row>
@@ -16250,7 +16283,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Malawi</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -16260,12 +16293,12 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>C/L — centre-right</t>
+          <t>C/L — centre-right security-oriented</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>R — centre-right</t>
+          <t>R — centre-right security-oriented</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -16282,7 +16315,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Malawi</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -16292,17 +16325,17 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>C/L — coalition/centrist</t>
+          <t>C/L — centre-right</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>L/C — coalition/centrist</t>
+          <t>R — centre-right</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
+          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
         </is>
       </c>
     </row>
@@ -16314,7 +16347,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Moldova</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -16324,12 +16357,12 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>C/L — liberal-centrist</t>
+          <t>C/L — coalition/centrist</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>L/C — liberal-centrist</t>
+          <t>L/C — coalition/centrist</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -16346,7 +16379,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Nepal</t>
+          <t>Moldova</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -16356,12 +16389,12 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>C/L — populist-centrist</t>
+          <t>C/L — liberal-centrist</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>L/C — populist-centrist</t>
+          <t>L/C — liberal-centrist</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -16378,7 +16411,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Nepal</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -16388,17 +16421,17 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>C/L — centre-right</t>
+          <t>C/L — populist-centrist</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>R — centre-right</t>
+          <t>L/C — populist-centrist</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
+          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
         </is>
       </c>
     </row>
@@ -16410,7 +16443,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Papua New Guinea</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -16420,17 +16453,17 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>C/L — developmental-centrist</t>
+          <t>C/L — centre-right</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>L/C — developmental-centrist</t>
+          <t>R — centre-right</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
+          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
         </is>
       </c>
     </row>
@@ -16442,7 +16475,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Papua New Guinea</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -16452,12 +16485,12 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>C/L — split executive</t>
+          <t>C/L — developmental-centrist</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>L/C — split executive</t>
+          <t>L/C — developmental-centrist</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -16474,7 +16507,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -16484,12 +16517,12 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>C/L — centrist caretaker</t>
+          <t>C/L — split executive</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>L/C — centrist caretaker</t>
+          <t>L/C — split executive</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -16506,7 +16539,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Saint Vincent and the Grenadines</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -16516,17 +16549,17 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>C/L — centre-right</t>
+          <t>C/L — centrist caretaker</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>R — centre-right</t>
+          <t>L/C — centrist caretaker</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
+          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
         </is>
       </c>
     </row>
@@ -16538,7 +16571,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Samoa</t>
+          <t>Saint Vincent and the Grenadines</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -16548,17 +16581,17 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>C/L — customary/centrist</t>
+          <t>C/L — centre-right</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>L/C — customary/centrist</t>
+          <t>R — centre-right</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
+          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
         </is>
       </c>
     </row>
@@ -16570,7 +16603,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>San Marino</t>
+          <t>Samoa</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -16580,12 +16613,12 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>C/L — centrist</t>
+          <t>C/L — customary/centrist</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>L/C — centrist</t>
+          <t>L/C — customary/centrist</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -16602,7 +16635,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>São Tomé and Príncipe</t>
+          <t>San Marino</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -16612,12 +16645,12 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>C/L — centre-right/centrist</t>
+          <t>C/L — centrist</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>L/C — centre-right/centrist</t>
+          <t>L/C — centrist</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -16634,7 +16667,7 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>São Tomé and Príncipe</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
@@ -16644,12 +16677,12 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>C/L — nationalist-developmental</t>
+          <t>C/L — centre-right/centrist</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>L/C — nationalist-developmental</t>
+          <t>L/C — centre-right/centrist</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -16666,7 +16699,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Solomon Islands</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -16676,17 +16709,17 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>C/L — centre-right/coalitional</t>
+          <t>C/L — nationalist-developmental</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>R — centre-right/coalitional</t>
+          <t>L/C — nationalist-developmental</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
+          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
         </is>
       </c>
     </row>
@@ -16698,7 +16731,7 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Solomon Islands</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -16708,17 +16741,17 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>C/L — coalition/centrist</t>
+          <t>C/L — centre-right/coalitional</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>L/C — coalition/centrist</t>
+          <t>R — centre-right/coalitional</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
+          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16763,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -16740,17 +16773,17 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>C/L — centre-right caretaker</t>
+          <t>C/L — coalition/centrist</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>R — centre-right caretaker</t>
+          <t>L/C — coalition/centrist</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
+          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
         </is>
       </c>
     </row>
@@ -16762,7 +16795,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -16772,17 +16805,17 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>C/L — consociational centre</t>
+          <t>C/L — centre-right caretaker</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>L/C — consociational centre</t>
+          <t>R — centre-right caretaker</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
+          <t>Label describes a centre-right/liberal market government without a conservative morphology; Methodology code R</t>
         </is>
       </c>
     </row>
@@ -16794,7 +16827,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Tanzania</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -16804,12 +16837,12 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>C/L — developmental-centrist</t>
+          <t>C/L — consociational centre</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>L/C — developmental-centrist</t>
+          <t>L/C — consociational centre</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -16826,7 +16859,7 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Timor-Leste</t>
+          <t>Tanzania</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -16836,12 +16869,12 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>C/L — nationalist-developmental</t>
+          <t>C/L — developmental-centrist</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>L/C — nationalist-developmental</t>
+          <t>L/C — developmental-centrist</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -16858,7 +16891,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Trinidad and Tobago</t>
+          <t>Timor-Leste</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -16868,12 +16901,12 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>C/L — centre-right/centrist</t>
+          <t>C/L — nationalist-developmental</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>L/C — centre-right/centrist</t>
+          <t>L/C — nationalist-developmental</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -16890,7 +16923,7 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Trinidad and Tobago</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
@@ -16900,12 +16933,12 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>C/L — wartime national-centrist</t>
+          <t>C/L — centre-right/centrist</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>L/C — wartime national-centrist</t>
+          <t>L/C — centre-right/centrist</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -16922,7 +16955,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -16932,12 +16965,12 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>C/L — liberal-centrist</t>
+          <t>C/L — wartime national-centrist</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>L/C — liberal-centrist</t>
+          <t>L/C — wartime national-centrist</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
@@ -16949,32 +16982,32 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Naming</t>
+          <t>C/L split</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Congo, Democratic Republic of the</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Country</t>
+          <t>Classification</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Congo, Democratic Republic of the</t>
+          <t>C/L — liberal-centrist</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Democratic Republic of the Congo</t>
+          <t>L/C — liberal-centrist</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>Use UN official short name</t>
+          <t>Label describes a centrist/developmental/coalitional/transitional government; Methodology says L/C is not coded primarily conservative</t>
         </is>
       </c>
     </row>
@@ -16986,7 +17019,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Congo, Republic of the</t>
+          <t>Congo, Democratic Republic of the</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -16996,12 +17029,12 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Congo, Republic of the</t>
+          <t>Congo, Democratic Republic of the</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Republic of the Congo</t>
+          <t>Democratic Republic of the Congo</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -17018,7 +17051,7 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Ivory Coast</t>
+          <t>Congo, Republic of the</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -17028,12 +17061,12 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Ivory Coast</t>
+          <t>Congo, Republic of the</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Côte d'Ivoire</t>
+          <t>Republic of the Congo</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
@@ -17050,7 +17083,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Micronesia</t>
+          <t>Ivory Coast</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -17060,12 +17093,12 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Micronesia</t>
+          <t>Ivory Coast</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Federated States of Micronesia</t>
+          <t>Côte d'Ivoire</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
@@ -17082,27 +17115,27 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Micronesia</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Head of state / government</t>
+          <t>Country</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Bongbong Marcos</t>
+          <t>Micronesia</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand "Bongbong" Marcos Jr.</t>
+          <t>Federated States of Micronesia</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>Full formal name</t>
+          <t>Use UN official short name</t>
         </is>
       </c>
     </row>
@@ -17114,27 +17147,27 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Head of state</t>
+          <t>Head of state / government</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Salman</t>
+          <t>Bongbong Marcos</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Salman bin Abdulaziz Al Saud</t>
+          <t>Ferdinand "Bongbong" Marcos Jr.</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>Full name for consistency</t>
+          <t>Full formal name</t>
         </is>
       </c>
     </row>
@@ -17146,32 +17179,64 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Head of state</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>Salman</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>Salman bin Abdulaziz Al Saud</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Full name for consistency</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Naming</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
           <t>Turkey</t>
         </is>
       </c>
-      <c r="C111" s="2" t="inlineStr">
+      <c r="C112" s="2" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="D111" s="2" t="inlineStr">
+      <c r="D112" s="2" t="inlineStr">
         <is>
           <t>Turkey</t>
         </is>
       </c>
-      <c r="E111" s="2" t="inlineStr">
+      <c r="E112" s="2" t="inlineStr">
         <is>
           <t>Türkiye</t>
         </is>
       </c>
-      <c r="F111" s="2" t="inlineStr">
+      <c r="F112" s="2" t="inlineStr">
         <is>
           <t>Use UN official short name</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F111"/>
+  <autoFilter ref="A1:F112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>